<commit_message>
chore: Update inventory template file for improved data management
</commit_message>
<xml_diff>
--- a/public/assets/templates/excel/template_location_inventory_wrm.xlsx
+++ b/public/assets/templates/excel/template_location_inventory_wrm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\project_warehouse\public\assets\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701B7A9D-8AA3-49A2-8546-415171AB1F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CA8EFA-EC4C-4922-9BE9-A00FACFC6E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>PLANT</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>ZONA</t>
+  </si>
+  <si>
+    <t>BIN</t>
   </si>
 </sst>
 </file>
@@ -59,7 +62,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -70,6 +73,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -95,6 +104,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
@@ -414,7 +424,7 @@
     <col min="10" max="11" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -427,6 +437,9 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>